<commit_message>
intel whole journey regressiont testing
</commit_message>
<xml_diff>
--- a/reports/link_check_production.xlsx
+++ b/reports/link_check_production.xlsx
@@ -495,14 +495,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,7 +538,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en</t>
+          <t>https://cartlow.com/uae/en</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
@@ -555,12 +555,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/set-country-locale?lang=ar&amp;country=uae</t>
+          <t>https://cartlow.com/customer/login</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>العربية</t>
+          <t>Sign up or Login</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -576,12 +576,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://tradein-buyback.cartlow.com/</t>
+          <t>https://cartlow.com/consumer-electronic</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Sell Your Device</t>
+          <t>Consumer Electronic</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -589,11 +589,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Sell Your Device</t>
-        </is>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -601,12 +597,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://cartlow.com/uae/en/search?criteria_id=543</t>
+          <t>https://cartlow.com/bundles</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Mobiles</t>
+          <t>Bundles</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -614,11 +610,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Mobiles</t>
-        </is>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -626,12 +618,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/secondary/home/perfumes</t>
+          <t>https://cartlow.com/patio-lawn-garden</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Original Perfumes 🔥</t>
+          <t>Patio, Lawn &amp; Garden</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -639,11 +631,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Original Perfumes 🔥</t>
-        </is>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -651,12 +639,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/secondary/home/gift-cards</t>
+          <t>https://cartlow.com/consumables</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Gift Cards</t>
+          <t>Consumables</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -664,11 +652,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Gift Cards</t>
-        </is>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -676,12 +660,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/tablets</t>
+          <t>https://cartlow.com/media-books</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Tablets</t>
+          <t>Media &amp; books</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -689,11 +673,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Tablets</t>
-        </is>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -701,12 +681,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/smartwatches</t>
+          <t>https://cartlow.com/home-lifestyle</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Smartwatches</t>
+          <t>Home &amp; Lifestyle</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -714,11 +694,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Smartwatches</t>
-        </is>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -726,12 +702,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/laptops</t>
+          <t>https://cartlow.com/fashion</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Laptops</t>
+          <t>Fashion</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -739,11 +715,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Laptops</t>
-        </is>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -751,12 +723,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/watches</t>
+          <t>https://cartlow.com/warranty</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Watches</t>
+          <t>Warranty</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -764,11 +736,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -776,12 +744,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/accessories</t>
+          <t>https://cartlow.com/warehouse-deal</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Electronic Accessories</t>
+          <t>Warehouse Deal</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -789,11 +757,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Electronic Accessories</t>
-        </is>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -801,12 +765,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/beauty</t>
+          <t>https://tradein-buyback.cartlow.com/</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Beauty</t>
+          <t>Sell your device</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -814,11 +778,7 @@
           <t>NAV</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Beauty</t>
-        </is>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -826,12 +786,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/sports</t>
+          <t>https://cartlow.com/set-country-locale?lang=ar&amp;country=uae</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Sports &amp; Play Gear</t>
+          <t>العربية</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -841,7 +801,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Sports &amp; Play Gear</t>
+          <t>العربية</t>
         </is>
       </c>
     </row>
@@ -851,24 +811,16 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://cartlow.com/uae/en/baby</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Baby</t>
-        </is>
-      </c>
+          <t>https://cartlow.com/customer/wishlist</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>NAV</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Baby</t>
-        </is>
-      </c>
+      <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -876,12 +828,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?criteria_id=973</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/sevices</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Home Appliances</t>
+          <t>Services &amp; Repair</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -891,7 +843,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Home Appliances</t>
+          <t>Services &amp; Repair</t>
         </is>
       </c>
     </row>
@@ -901,20 +853,24 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=apple+devices</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/mobiles-uae</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>See All</t>
+          <t>Mobiles</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Mobiles</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -922,20 +878,24 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=apple+iphone</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/perfumes</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>iPhones</t>
+          <t>Original Perfumes</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Original Perfumes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -943,20 +903,24 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=apple+watches&amp;categories=12019&amp;brand=39</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/gift-cards</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Apple Watches</t>
+          <t>Gift Cards</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Gift Cards</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -964,20 +928,24 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=macbook&amp;brand=39</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/tablets-uae</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Macbook</t>
+          <t>Tablets</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Tablets</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -985,20 +953,24 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=ipads&amp;brand=39</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/smartwatches-uae</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>iPads</t>
+          <t>Smartwatches</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Smartwatches</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1006,20 +978,24 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=imac&amp;brand=39</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/laptops-uae</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>iMac</t>
+          <t>Laptops</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Laptops</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1027,20 +1003,24 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?criteria_id=10</t>
+          <t>https://www.cartlow.com/uae/en/secondary/home/gg-store-l2-page</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>See All</t>
+          <t>Beauty</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Beauty</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1048,20 +1028,24 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=binance+gift+cards&amp;brand=5095</t>
+          <t>https://cartlow.com/uae/en/secondary/home/gaming</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Gaming</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1069,20 +1053,24 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=binance+gift+cards&amp;brand=1742%2C5091%2C5186%2C2013%2C1392%2C5094%2C248=5095</t>
+          <t>https://www.cartlow.com/uae/en/sports</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Games</t>
+          <t>Sports &amp; Play Gear</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Sports &amp; Play Gear</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1090,20 +1078,24 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?criteria_id=943</t>
+          <t>https://cartlow.com/uae/en/baby</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Online Shopping</t>
+          <t>Baby</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Baby</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1111,20 +1103,24 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?criteria_id=942</t>
+          <t>https://cartlow.com/uae/en/secondary/home/home-appliances-uae</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Telcos</t>
+          <t>Home Appliances</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr"/>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Home Appliances</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1132,17 +1128,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?criteria_id=466</t>
+          <t>https://wholesale.cartlow.com</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Digital Entertainment</t>
+          <t>Wholesale</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>FOOTER</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr"/>
@@ -1153,12 +1149,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?criteria_id=16</t>
+          <t>https://www.cartlow.com/uae/en/search?query=apple+devices</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>See all</t>
+          <t>See All</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1174,12 +1170,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=Dell+Laptops</t>
+          <t>https://www.cartlow.com/uae/en/search?query=apple+iphone</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Dell</t>
+          <t>iPhones</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1195,12 +1191,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=lenovo+Laptops</t>
+          <t>https://www.cartlow.com/uae/en/search?query=apple+watches&amp;categories=12019&amp;brand=39</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Lenovo</t>
+          <t>Apple Watches</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1216,12 +1212,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=HP+Laptops</t>
+          <t>https://www.cartlow.com/uae/en/search?query=macbook&amp;brand=39</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Macbook</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1237,12 +1233,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=acer+Laptops</t>
+          <t>https://www.cartlow.com/uae/en/search?query=ipads&amp;brand=39</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Acer</t>
+          <t>iPads</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1258,12 +1254,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=mo%5Cicrosoft+Laptops</t>
+          <t>https://www.cartlow.com/uae/en/search?query=imac&amp;brand=39</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>iMac</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1279,7 +1275,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=gaming</t>
+          <t>https://www.cartlow.com/uae/en/search?criteria_id=10</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1300,12 +1296,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=Gaming+desktop+&amp;conditions=32</t>
+          <t>https://www.cartlow.com/uae/en/search?query=binance+gift+cards&amp;brand=5095</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Gaming PCs</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1321,12 +1317,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=Gaming+Monitor&amp;categories=16002</t>
+          <t>https://www.cartlow.com/uae/en/search?query=binance+gift+cards&amp;brand=1742%2C5091%2C5186%2C2013%2C1392%2C5094%2C248=5095</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Gaming Monitors</t>
+          <t>Games</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1342,12 +1338,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=Consoles</t>
+          <t>https://www.cartlow.com/uae/en/search?criteria_id=943</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Consoles</t>
+          <t>Online Shopping</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1363,12 +1359,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=headset</t>
+          <t>https://www.cartlow.com/uae/en/search?criteria_id=942</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Headset</t>
+          <t>Telecommunication</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1384,12 +1380,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/search?query=keyboard+and+mouse+gaming&amp;conditions=32&amp;categories=16010</t>
+          <t>https://www.cartlow.com/uae/en/search?criteria_id=466</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Gaming Keyboard &amp; Mice</t>
+          <t>Digital Entertainment</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1405,12 +1401,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/about-us</t>
+          <t>https://www.cartlow.com/uae/en/search?criteria_id=16</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>About Company</t>
+          <t>See all</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1426,12 +1422,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/our-story</t>
+          <t>https://www.cartlow.com/uae/en/search?query=Dell+Laptops</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Cartlow’s Journey</t>
+          <t>Dell</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1447,12 +1443,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/careers</t>
+          <t>https://www.cartlow.com/uae/en/search?query=lenovo+Laptops</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Careers</t>
+          <t>Lenovo</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1468,10 +1464,14 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>https://twitter.com/CartlowUAE?t=T7E2shWf2JTql15OwSvmNw&amp;s=08</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr"/>
+          <t>https://www.cartlow.com/uae/en/search?query=HP+Laptops</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1480,21 +1480,25 @@
       <c r="E44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/cartlowuae?mibextid=ZbWKwL</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr"/>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr"/>
+      <c r="A45" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/search?query=acer+Laptops</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Acer</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -1502,10 +1506,14 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>https://instagram.com/cartlowuae?igshid=MzRlODBiNWFlZA==</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr"/>
+          <t>https://www.cartlow.com/uae/en/search?query=mo%5Cicrosoft+Laptops</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1519,10 +1527,14 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>https://linkedin.com/company/cartlow</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr"/>
+          <t>https://www.cartlow.com/uae/en/search?query=gaming</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>See All</t>
+        </is>
+      </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1536,10 +1548,14 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cartlowofficial</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr"/>
+          <t>https://www.cartlow.com/uae/en/search?query=Gaming+desktop+&amp;conditions=32</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Gaming PCs</t>
+        </is>
+      </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1553,10 +1569,14 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>https://play.google.com/store/apps/details?id=com.cartlow.android&amp;hl=en</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr"/>
+          <t>https://www.cartlow.com/uae/en/search?query=Gaming+Monitor&amp;categories=16002</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Gaming Monitors</t>
+        </is>
+      </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1570,10 +1590,14 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>https://apps.apple.com/ae/app/cartlow/id1455009311</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr"/>
+          <t>https://www.cartlow.com/uae/en/search?query=Consoles</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Consoles</t>
+        </is>
+      </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1587,12 +1611,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/contact-us</t>
+          <t>https://www.cartlow.com/uae/en/search?query=headset</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Contact Us</t>
+          <t>Headset</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1608,12 +1632,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/faqs</t>
+          <t>https://www.cartlow.com/uae/en/search?query=keyboard+and+mouse+gaming&amp;conditions=32&amp;categories=16010</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>FAQs</t>
+          <t>Gaming Keyboard &amp; Mice</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -1629,12 +1653,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/complaints-and-suggestions</t>
+          <t>https://www.cartlow.com/uae/en/page/about-us</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Complaints &amp; Suggestions</t>
+          <t>About Company</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -1650,12 +1674,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/track-order</t>
+          <t>https://www.cartlow.com/uae/en/page/our-story</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Track Your Order</t>
+          <t>Cartlow’s Journey</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1671,12 +1695,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>https://wholesale.cartlow.com/</t>
+          <t>https://www.cartlow.com/uae/en/page/careers</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Cartlow Wholesale</t>
+          <t>Careers</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1692,14 +1716,10 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>https://mobocheck.com/</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Mobocheck</t>
-        </is>
-      </c>
+          <t>https://twitter.com/CartlowUAE?t=T7E2shWf2JTql15OwSvmNw&amp;s=08</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr"/>
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1708,25 +1728,21 @@
       <c r="E56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>https://www.ardroid.com/</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Ardroid</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr"/>
+      <c r="A57" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/cartlowuae?mibextid=ZbWKwL</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -1734,14 +1750,10 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/shipping-policy</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Shipping</t>
-        </is>
-      </c>
+          <t>https://instagram.com/cartlowuae?igshid=MzRlODBiNWFlZA==</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1755,14 +1767,10 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/payment-policy</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
+          <t>https://linkedin.com/company/cartlow</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr"/>
       <c r="D59" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1776,14 +1784,10 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/marketing-tools</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>Marketing Solutions</t>
-        </is>
-      </c>
+          <t>https://www.tiktok.com/@cartlowofficial</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr"/>
       <c r="D60" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1797,14 +1801,10 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/strategic-and-logistical-services-tools</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>Strategic &amp; Logistical Services</t>
-        </is>
-      </c>
+          <t>https://play.google.com/store/apps/details?id=com.cartlow.android&amp;hl=en</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr"/>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1818,14 +1818,10 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/seller</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Sell with Cartlow</t>
-        </is>
-      </c>
+          <t>https://apps.apple.com/ae/app/cartlow/id1455009311</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr"/>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>FOOTER</t>
@@ -1839,12 +1835,12 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/why-expand-with-cartlow</t>
+          <t>https://www.cartlow.com/contact-us</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Why Expand with Cartlow?</t>
+          <t>Contact Us</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -1860,12 +1856,12 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/pricing</t>
+          <t>https://www.cartlow.com/uae/en/page/faqs</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>FAQs</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -1881,12 +1877,12 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/advertise-your-products</t>
+          <t>https://www.cartlow.com/uae/en/page/complaints-and-suggestions</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Advertise Your Products</t>
+          <t>Complaints &amp; Suggestions</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
@@ -1902,12 +1898,12 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/terms-conditions</t>
+          <t>https://www.cartlow.com/uae/en/page/track-order</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Terms &amp; Conditions</t>
+          <t>Track Your Order</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -1923,12 +1919,12 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/privacy-policy</t>
+          <t>https://wholesale.cartlow.com/</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Privacy Policy</t>
+          <t>Cartlow Wholesale</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -1944,12 +1940,12 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/refund-policy</t>
+          <t>https://mobocheck.com/</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Refund Policy</t>
+          <t>Mobocheck</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -1965,12 +1961,12 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/return-policy</t>
+          <t>https://www.ardroid.com/</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Return Policy</t>
+          <t>Ardroid</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -1986,12 +1982,12 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/warranty-policy</t>
+          <t>https://www.cartlow.com/uae/en/page/shipping-policy</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Warranty Policy</t>
+          <t>Shipping</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -2007,12 +2003,12 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/cashback-policy</t>
+          <t>https://www.cartlow.com/uae/en/page/payment-policy</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Cashback Policy</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -2028,12 +2024,12 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/user-data-rights</t>
+          <t>https://www.cartlow.com/uae/en/page/marketing-tools</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>User Data Rights</t>
+          <t>Marketing Solutions</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2049,12 +2045,12 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>https://www.cartlow.com/uae/en/page/third-party-services-disclosure</t>
+          <t>https://www.cartlow.com/uae/en/page/strategic-and-logistical-services-tools</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Third Party Services Disclosure</t>
+          <t>Strategic &amp; Logistical Services</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2070,16 +2066,268 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
+          <t>https://www.cartlow.com/seller</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Sell with Cartlow</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/why-expand-with-cartlow</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Why Expand with Cartlow?</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/pricing</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/advertise-your-products</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Advertise Your Products</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/terms-conditions</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Terms &amp; Conditions</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/privacy-policy</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Privacy Policy</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/refund-policy</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Refund Policy</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/return-policy</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Return Policy</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/warranty-policy</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Warranty Policy</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/cashback-policy</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Cashback Policy</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/user-data-rights</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>User Data Rights</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cartlow.com/uae/en/page/third-party-services-disclosure</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Third Party Services Disclosure</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
           <t>https://www.cartlow.com/uae/en/</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr"/>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>FOOTER</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>FOOTER</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
         <is>
           <t>Deliver to</t>
         </is>

</xml_diff>